<commit_message>
Update roster: Export Roster May 2026 Version 3.xlsx
</commit_message>
<xml_diff>
--- a/rosters/.versions/2026-05/current.xlsx
+++ b/rosters/.versions/2026-05/current.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://omanair-my.sharepoint.com/personal/80235_hq_omanair_com/Documents/Desktop/Rosters/STAFF OPERATION SCHEDULE/ROSTER 2026/OPS/05 May/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://omanair-my.sharepoint.com/personal/80235_hq_omanair_com/Documents/Desktop/Rosters/STAFF OPERATION SCHEDULE/Roster with 2 OFF/05 May26/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FC67CAF7-2C87-451A-9C76-36015329D2FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{DBFD20C6-21BE-4A98-9DB3-DBC523CCAF17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{9736B67C-D61B-41E1-B07B-429B3D8AE9CC}"/>
   </bookViews>
@@ -75,7 +75,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="J9" authorId="0" shapeId="0" xr:uid="{F6F20C50-A605-42D8-A2AA-A9C471664108}">
+    <comment ref="J9" authorId="0" shapeId="0" xr:uid="{03BEC542-DC83-4484-9ED4-997CD07222FC}">
       <text>
         <r>
           <rPr>
@@ -99,7 +99,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q13" authorId="0" shapeId="0" xr:uid="{E0BCA8CB-4007-4498-85F3-C93DEB09C944}">
+    <comment ref="Q13" authorId="0" shapeId="0" xr:uid="{46FBE38B-C63E-403A-B55D-6B9F3FE326E0}">
       <text>
         <r>
           <rPr>
@@ -123,7 +123,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R14" authorId="0" shapeId="0" xr:uid="{66C96275-281B-46B0-8EDC-D0FAA3B9904A}">
+    <comment ref="R14" authorId="0" shapeId="0" xr:uid="{CF48607F-190E-4360-B9C2-5902E365E994}">
       <text>
         <r>
           <rPr>
@@ -147,7 +147,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S14" authorId="0" shapeId="0" xr:uid="{FC31F6AA-5901-4BED-8712-ECF0513317CB}">
+    <comment ref="S14" authorId="0" shapeId="0" xr:uid="{28BF2ABC-12A7-43E1-A093-A9CCDE47CBB2}">
       <text>
         <r>
           <rPr>
@@ -171,7 +171,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q15" authorId="0" shapeId="0" xr:uid="{7128C0C4-5B55-4DA9-B6EF-34CD410BF5E8}">
+    <comment ref="Q15" authorId="0" shapeId="0" xr:uid="{3315337E-3DF1-48CB-8F0D-CBC24EDED16D}">
       <text>
         <r>
           <rPr>
@@ -195,7 +195,31 @@
         </r>
       </text>
     </comment>
-    <comment ref="R21" authorId="0" shapeId="0" xr:uid="{C61CEACE-7040-4713-99F0-0FDE0618727D}">
+    <comment ref="AG20" authorId="0" shapeId="0" xr:uid="{6BC994B4-4A44-41A1-A510-3EFA13F518DE}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Acting Supervisor on behalf of Jay</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R21" authorId="0" shapeId="0" xr:uid="{37B724C9-959E-4F45-AA47-E1F62744E51F}">
       <text>
         <r>
           <rPr>
@@ -219,7 +243,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S21" authorId="0" shapeId="0" xr:uid="{D9752FC4-0BF5-40FB-A13D-86BBE7334FD8}">
+    <comment ref="S21" authorId="0" shapeId="0" xr:uid="{0AF407EE-5F60-4B25-9E6D-75885E2E7C8B}">
       <text>
         <r>
           <rPr>
@@ -243,7 +267,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="O22" authorId="0" shapeId="0" xr:uid="{6B4BE2A2-5AC1-4A78-843C-12AC66CC145B}">
+    <comment ref="O22" authorId="0" shapeId="0" xr:uid="{F9628C7F-42EE-4011-94F9-30AE0C672026}">
       <text>
         <r>
           <rPr>
@@ -267,7 +291,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q22" authorId="0" shapeId="0" xr:uid="{C3283DF1-81E0-41F1-8846-09377BE38E17}">
+    <comment ref="Q22" authorId="0" shapeId="0" xr:uid="{ABEE8D00-4A2D-473C-99D5-AB7866D35BB5}">
       <text>
         <r>
           <rPr>
@@ -291,7 +315,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K26" authorId="0" shapeId="0" xr:uid="{E859518D-09AA-486C-910D-9D3B988C377C}">
+    <comment ref="K26" authorId="0" shapeId="0" xr:uid="{285B9D9A-FA8B-47A1-8E50-926F8399D184}">
       <text>
         <r>
           <rPr>
@@ -315,7 +339,55 @@
         </r>
       </text>
     </comment>
-    <comment ref="R28" authorId="0" shapeId="0" xr:uid="{DF0916D2-E5A2-4218-891F-4ABBBFFBB256}">
+    <comment ref="AF26" authorId="0" shapeId="0" xr:uid="{FE8BA395-F598-407C-8CC0-491230DD84A3}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Acting Supervisor on behalf of Saleh</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AG26" authorId="0" shapeId="0" xr:uid="{4CCA8B84-D955-452E-95E1-5DFF83C03464}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Acting supervisor on behal of Saleh</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R28" authorId="0" shapeId="0" xr:uid="{4B4DE37F-31B3-4467-9DD7-37E35B9BEC13}">
       <text>
         <r>
           <rPr>
@@ -339,7 +411,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S28" authorId="0" shapeId="0" xr:uid="{C366D4EC-DDDA-49FB-8537-075E80C04E0B}">
+    <comment ref="S28" authorId="0" shapeId="0" xr:uid="{8EF7370A-0FCF-46B5-8B93-4986CBF7223A}">
       <text>
         <r>
           <rPr>
@@ -363,7 +435,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L29" authorId="0" shapeId="0" xr:uid="{F137B47C-D25B-464D-A7D7-F4A3EDC2E809}">
+    <comment ref="L29" authorId="0" shapeId="0" xr:uid="{DC35BEEB-8106-4955-9805-DB6835781714}">
       <text>
         <r>
           <rPr>
@@ -387,7 +459,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="F30" authorId="0" shapeId="0" xr:uid="{41100FCF-8FD1-455B-B6FF-A5645C9267D4}">
+    <comment ref="F30" authorId="0" shapeId="0" xr:uid="{754C5C68-8FBE-44D9-BBFB-0DBEE584F5AA}">
       <text>
         <r>
           <rPr>
@@ -411,7 +483,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="R34" authorId="0" shapeId="0" xr:uid="{7123E160-215B-4092-9E28-94EF6C674DDE}">
+    <comment ref="R34" authorId="0" shapeId="0" xr:uid="{A568837D-93E4-4B89-9E44-448C7C6BCA63}">
       <text>
         <r>
           <rPr>
@@ -435,7 +507,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L35" authorId="0" shapeId="0" xr:uid="{DBF514ED-8141-4102-800C-0D83CA5406E0}">
+    <comment ref="L35" authorId="0" shapeId="0" xr:uid="{CA25FACE-C0AE-4562-94B3-EFD10817D144}">
       <text>
         <r>
           <rPr>
@@ -459,7 +531,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q38" authorId="0" shapeId="0" xr:uid="{5E90E177-ED20-4E93-8F77-3B370CE9BF97}">
+    <comment ref="Q38" authorId="0" shapeId="0" xr:uid="{F49E7344-76A7-4E6E-8063-D8858D900FC9}">
       <text>
         <r>
           <rPr>
@@ -483,7 +555,55 @@
         </r>
       </text>
     </comment>
-    <comment ref="R43" authorId="0" shapeId="0" xr:uid="{DD1A518C-6974-4B57-BEFF-92E86142C16F}">
+    <comment ref="R41" authorId="0" shapeId="0" xr:uid="{25F4F0D6-9086-47FD-8565-D3B6F7D2E201}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+CWO</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S41" authorId="0" shapeId="0" xr:uid="{605185C3-B2F1-445E-81D2-43F7C1A86487}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+CWO</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R43" authorId="0" shapeId="0" xr:uid="{C382CFB7-A510-40D2-BDD4-E92BF1068149}">
       <text>
         <r>
           <rPr>
@@ -507,7 +627,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S43" authorId="0" shapeId="0" xr:uid="{2E511B3E-1587-4012-B93D-E44E8CC3B2E2}">
+    <comment ref="S43" authorId="0" shapeId="0" xr:uid="{D2048226-EED6-48E7-A244-D6FF9B0AFE81}">
       <text>
         <r>
           <rPr>
@@ -531,7 +651,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="W44" authorId="0" shapeId="0" xr:uid="{80B6D286-9324-4CBB-9947-8E3F01B720D3}">
+    <comment ref="W44" authorId="0" shapeId="0" xr:uid="{7DE6BFB3-C33A-460F-B796-20485E232123}">
       <text>
         <r>
           <rPr>
@@ -555,7 +675,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q45" authorId="0" shapeId="0" xr:uid="{C80E8B0A-D365-4C98-A1AA-95B0329F5643}">
+    <comment ref="Q45" authorId="0" shapeId="0" xr:uid="{E6D8F30A-C851-4974-BEEE-EA52D999CE82}">
       <text>
         <r>
           <rPr>
@@ -579,7 +699,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="L47" authorId="0" shapeId="0" xr:uid="{817C78B9-460A-4C6C-8E18-2F7873EC6665}">
+    <comment ref="L47" authorId="0" shapeId="0" xr:uid="{B721E896-6A72-438B-837C-4763C2906E18}">
       <text>
         <r>
           <rPr>
@@ -603,7 +723,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="K48" authorId="0" shapeId="0" xr:uid="{DC150764-0495-4EC4-BEF1-CA288921D67D}">
+    <comment ref="K48" authorId="0" shapeId="0" xr:uid="{D7E5170E-8069-4823-BCED-B8344CAB7B27}">
       <text>
         <r>
           <rPr>
@@ -627,7 +747,127 @@
         </r>
       </text>
     </comment>
-    <comment ref="R48" authorId="0" shapeId="0" xr:uid="{E11B68D7-0BF6-4ECD-B540-859FE69E1C06}">
+    <comment ref="Q49" authorId="0" shapeId="0" xr:uid="{7B4F57D4-742E-433F-BAA9-497CBE46DFFB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+LAR</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="Y49" authorId="0" shapeId="0" xr:uid="{508DE0A1-409A-4F67-92E0-788D70D6E683}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+ADP</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F51" authorId="0" shapeId="0" xr:uid="{C9EE535B-A15B-4720-AF0A-355B8A49EB2E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+OT</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="G51" authorId="0" shapeId="0" xr:uid="{0E6A6AD4-C137-49AA-95F6-E6FD09D467EC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+OT</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="L55" authorId="0" shapeId="0" xr:uid="{CD15FE75-7A3D-477F-997B-F46D1C6DAB58}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+SMS</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="R55" authorId="0" shapeId="0" xr:uid="{5EB529AC-91B7-4E7E-BFFD-06A3F211912B}">
       <text>
         <r>
           <rPr>
@@ -651,7 +891,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="S48" authorId="0" shapeId="0" xr:uid="{90187567-65E1-414F-B318-B42A60485352}">
+    <comment ref="S55" authorId="0" shapeId="0" xr:uid="{3424F110-5CB4-441F-8D69-AB35A70456BE}">
       <text>
         <r>
           <rPr>
@@ -675,7 +915,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Q49" authorId="0" shapeId="0" xr:uid="{93D1B246-AC46-43A0-AFFA-C69FDBC14E13}">
+    <comment ref="Q61" authorId="0" shapeId="0" xr:uid="{5809084B-3738-4EC5-A4B9-1AA706451FF1}">
       <text>
         <r>
           <rPr>
@@ -699,175 +939,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="Y49" authorId="0" shapeId="0" xr:uid="{D0891FAA-32CE-48AA-BA98-CDA21C8A72EC}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Rodolfo C Magcaling:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-ADP</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="F51" authorId="0" shapeId="0" xr:uid="{A016C86E-29DC-46A8-B715-3BB94E6356C1}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Rodolfo C Magcaling:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-OT</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="G51" authorId="0" shapeId="0" xr:uid="{9794953C-2ACE-4B10-92B0-BE8E32AC8A90}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Rodolfo C Magcaling:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-OT</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="L55" authorId="0" shapeId="0" xr:uid="{AC439B05-80A0-4BA1-A50D-CF1571C1632F}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Rodolfo C Magcaling:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-SMS</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R55" authorId="0" shapeId="0" xr:uid="{AF28AB55-9467-4F1C-BF93-0024F0DF3B96}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Rodolfo C Magcaling:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-CWO</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="S55" authorId="0" shapeId="0" xr:uid="{137DF81B-2631-437F-A937-C4A5848E5A77}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Rodolfo C Magcaling:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-CWO</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="Q61" authorId="0" shapeId="0" xr:uid="{34CE854F-E4DE-4AA4-8F48-5EDA718E61D9}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Rodolfo C Magcaling:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-LAR</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="P81" authorId="0" shapeId="0" xr:uid="{4E7005B8-7BC5-494C-AF73-E9B435262701}">
+    <comment ref="P81" authorId="0" shapeId="0" xr:uid="{27FE63B1-B5FC-44CA-820F-9F0148694609}">
       <text>
         <r>
           <rPr>
@@ -1056,6 +1128,30 @@
         </r>
       </text>
     </comment>
+    <comment ref="AG10" authorId="0" shapeId="0" xr:uid="{AE64D879-E0EB-4292-BC75-565D14F9E110}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Acting Supervisor on behalf of Jay</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="R11" authorId="0" shapeId="0" xr:uid="{1AAB0E81-08AE-4474-ACA3-9427AC3DD4EB}">
       <text>
         <r>
@@ -1173,6 +1269,54 @@
           </rPr>
           <t xml:space="preserve">
 Forklift</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AF16" authorId="0" shapeId="0" xr:uid="{D9D5DFDC-44E5-40E6-B7D6-A8E4F159C880}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Acting Supervisor on behalf of Saleh</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="AG16" authorId="0" shapeId="0" xr:uid="{2110C9C0-4DAC-4FFD-97E9-FCDB1773CFB4}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Acting supervisor on behal of Saleh</t>
         </r>
       </text>
     </comment>
@@ -1354,6 +1498,54 @@
         </r>
       </text>
     </comment>
+    <comment ref="R16" authorId="0" shapeId="0" xr:uid="{1D16DBAC-7518-4025-82AC-8B78815326FB}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+CWO</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="S16" authorId="0" shapeId="0" xr:uid="{74239DB6-C0A5-419C-8861-EE40F72743DC}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Rodolfo C Magcaling:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+CWO</t>
+        </r>
+      </text>
+    </comment>
     <comment ref="R18" authorId="0" shapeId="0" xr:uid="{D42098F5-5F14-489A-A930-521A47753876}">
       <text>
         <r>
@@ -1495,54 +1687,6 @@
           </rPr>
           <t xml:space="preserve">
 Forklift</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="R23" authorId="0" shapeId="0" xr:uid="{9CDED2D9-35A3-464A-A62A-8332D081FFA6}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Rodolfo C Magcaling:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-CWO</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="S23" authorId="0" shapeId="0" xr:uid="{1E11B87D-F440-4735-B152-1ECABBFAA402}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>Rodolfo C Magcaling:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-CWO</t>
         </r>
       </text>
     </comment>
@@ -2502,7 +2646,7 @@
     <numFmt numFmtId="165" formatCode="dd\-mm\-yyyy"/>
     <numFmt numFmtId="166" formatCode="dd"/>
   </numFmts>
-  <fonts count="21" x14ac:knownFonts="1">
+  <fonts count="23" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -2655,6 +2799,19 @@
       <color indexed="81"/>
       <name val="Tahoma"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="13">
@@ -4152,7 +4309,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="230">
+  <dxfs count="175">
     <dxf>
       <font>
         <color auto="1"/>
@@ -4558,587 +4715,6 @@
       <fill>
         <patternFill>
           <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor auto="1"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor auto="1"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFF0000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <fgColor auto="1"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5893,9 +5469,33 @@
       </fill>
     </dxf>
     <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <fgColor auto="1"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
       <fill>
         <patternFill>
           <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5915,7 +5515,74 @@
       </font>
       <fill>
         <patternFill>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
           <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="0" tint="-0.14996795556505021"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color auto="1"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFC00000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -5962,16 +5629,6 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
           <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
@@ -5982,7 +5639,14 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="8" tint="0.39994506668294322"/>
+          <bgColor theme="7" tint="0.39994506668294322"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="8" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6053,33 +5717,6 @@
       <fill>
         <patternFill>
           <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFC00000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="8" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6209,16 +5846,6 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
           <bgColor theme="9" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
@@ -6237,16 +5864,6 @@
       <fill>
         <patternFill>
           <bgColor theme="0" tint="-0.14996795556505021"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6282,11 +5899,11 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="0"/>
+        <color auto="1"/>
       </font>
       <fill>
         <patternFill>
-          <bgColor rgb="FFFF0000"/>
+          <bgColor theme="4" tint="0.39994506668294322"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6296,8 +5913,17 @@
       </font>
       <fill>
         <patternFill>
-          <fgColor auto="1"/>
-          <bgColor theme="5" tint="0.59996337778862885"/>
+          <bgColor rgb="FF7030A0"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF0000"/>
         </patternFill>
       </fill>
     </dxf>
@@ -6327,17 +5953,8 @@
       </font>
       <fill>
         <patternFill>
-          <bgColor theme="4" tint="0.39994506668294322"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color auto="1"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF7030A0"/>
+          <fgColor auto="1"/>
+          <bgColor theme="5" tint="0.59996337778862885"/>
         </patternFill>
       </fill>
     </dxf>
@@ -12377,26 +11994,26 @@
     <mergeCell ref="X4:Z4"/>
   </mergeCells>
   <conditionalFormatting sqref="E8:AI37 AK8:AN37 E39:AI42">
-    <cfRule type="expression" dxfId="229" priority="4">
+    <cfRule type="expression" dxfId="174" priority="4">
       <formula>LEFT(E8,1)="N"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="228" priority="5">
+    <cfRule type="expression" dxfId="173" priority="5">
       <formula>LEFT(E8,1)="A"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="227" priority="7">
+    <cfRule type="expression" dxfId="172" priority="7">
       <formula>LEFT(E8,1)="M"</formula>
     </cfRule>
-    <cfRule type="expression" dxfId="226" priority="8">
+    <cfRule type="expression" dxfId="171" priority="8">
       <formula>LEFT(E8,1)="D"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E39:AI42 E8:AI37 AK8:AN37">
-    <cfRule type="expression" dxfId="225" priority="3">
+    <cfRule type="expression" dxfId="170" priority="3">
       <formula>LEFT(E8,1)="O"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E39:AI42">
-    <cfRule type="expression" dxfId="224" priority="1">
+    <cfRule type="expression" dxfId="169" priority="1">
       <formula>ISEVEN(ROW($E39))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -13392,16 +13009,16 @@
         <v>223</v>
       </c>
       <c r="AF10" s="50" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="AG10" s="50" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="AH10" s="50" t="s">
         <v>199</v>
       </c>
       <c r="AI10" s="50" t="s">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="AJ10" s="50" t="s">
         <v>222</v>
@@ -13412,15 +13029,15 @@
       </c>
       <c r="AM10" s="49">
         <f t="shared" si="6"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AN10" s="49">
         <f t="shared" si="7"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AO10" s="49">
         <f t="shared" si="8"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP10" s="49">
         <f t="shared" si="9"/>
@@ -13511,19 +13128,19 @@
         <v>223</v>
       </c>
       <c r="AE11" s="50" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="AF11" s="50" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AG11" s="50" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AH11" s="50" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="AI11" s="50" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="AJ11" s="50" t="s">
         <v>223</v>
@@ -13534,15 +13151,15 @@
       </c>
       <c r="AM11" s="49">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AN11" s="49">
         <f t="shared" si="7"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AO11" s="49">
         <f t="shared" si="8"/>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AP11" s="49">
         <f t="shared" si="9"/>
@@ -13645,7 +13262,7 @@
         <v>198</v>
       </c>
       <c r="AI12" s="50" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AJ12" s="50" t="s">
         <v>199</v>
@@ -13656,11 +13273,11 @@
       </c>
       <c r="AM12" s="49">
         <f t="shared" si="6"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AN12" s="49">
         <f t="shared" si="7"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AO12" s="49">
         <f t="shared" si="8"/>
@@ -14076,13 +13693,13 @@
         <v>198</v>
       </c>
       <c r="O16" s="50" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="P16" s="87" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="Q16" s="50" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="R16" s="50" t="s">
         <v>222</v>
@@ -14151,11 +13768,11 @@
       </c>
       <c r="AN16" s="49">
         <f t="shared" ref="AN16:AN29" si="12">COUNTIF($F16:$AJ16,"A*")</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AO16" s="49">
         <f t="shared" ref="AO16:AO29" si="13">COUNTIF($F16:$AJ16,"N*")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AP16" s="49">
         <f t="shared" ref="AP16:AP29" si="14">COUNTIF($F16:$AJ16,"O*")</f>
@@ -14322,7 +13939,7 @@
         <v>199</v>
       </c>
       <c r="O18" s="50" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="P18" s="50" t="s">
         <v>222</v>
@@ -14397,11 +14014,11 @@
       </c>
       <c r="AN18" s="49">
         <f t="shared" si="12"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AO18" s="49">
         <f t="shared" si="13"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AP18" s="49">
         <f t="shared" si="14"/>
@@ -14478,7 +14095,7 @@
         <v>198</v>
       </c>
       <c r="Z19" s="50" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AA19" s="50" t="s">
         <v>199</v>
@@ -14516,11 +14133,11 @@
       </c>
       <c r="AM19" s="49">
         <f t="shared" si="11"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AN19" s="49">
         <f t="shared" si="12"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AO19" s="49">
         <f t="shared" si="13"/>
@@ -14619,7 +14236,7 @@
         <v>198</v>
       </c>
       <c r="AF20" s="111" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AG20" s="111" t="s">
         <v>199</v>
@@ -14639,11 +14256,11 @@
       </c>
       <c r="AM20" s="49">
         <f t="shared" si="11"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AN20" s="49">
         <f t="shared" si="12"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AO20" s="49">
         <f t="shared" si="13"/>
@@ -15063,7 +14680,7 @@
         <v>199</v>
       </c>
       <c r="P24" s="50" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="Q24" s="50" t="s">
         <v>222</v>
@@ -15135,11 +14752,11 @@
       </c>
       <c r="AN24" s="49">
         <f t="shared" si="12"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AO24" s="49">
         <f t="shared" si="13"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AP24" s="49">
         <f t="shared" si="14"/>
@@ -15336,19 +14953,19 @@
         <v>223</v>
       </c>
       <c r="Y26" s="50" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="Z26" s="50" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="AA26" s="50" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AB26" s="50" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AC26" s="87" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="AD26" s="87" t="s">
         <v>223</v>
@@ -15377,15 +14994,15 @@
       </c>
       <c r="AM26" s="49">
         <f t="shared" si="11"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AN26" s="49">
         <f t="shared" si="12"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AO26" s="49">
         <f t="shared" si="13"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AP26" s="49">
         <f t="shared" si="14"/>
@@ -15459,7 +15076,7 @@
         <v>198</v>
       </c>
       <c r="Y27" s="50" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Z27" s="50" t="s">
         <v>199</v>
@@ -15480,7 +15097,7 @@
         <v>198</v>
       </c>
       <c r="AF27" s="111" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AG27" s="111" t="s">
         <v>199</v>
@@ -15500,11 +15117,11 @@
       </c>
       <c r="AM27" s="49">
         <f t="shared" si="11"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AN27" s="49">
         <f t="shared" si="12"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AO27" s="49">
         <f t="shared" si="13"/>
@@ -17149,10 +16766,10 @@
         <v>223</v>
       </c>
       <c r="R41" s="50" t="s">
-        <v>198</v>
+        <v>126</v>
       </c>
       <c r="S41" s="50" t="s">
-        <v>198</v>
+        <v>126</v>
       </c>
       <c r="T41" s="50" t="s">
         <v>199</v>
@@ -17211,7 +16828,7 @@
       </c>
       <c r="AM41" s="49">
         <f t="shared" si="16"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AN41" s="49">
         <f t="shared" si="17"/>
@@ -18003,10 +17620,10 @@
         <v>223</v>
       </c>
       <c r="R48" s="50" t="s">
-        <v>126</v>
+        <v>198</v>
       </c>
       <c r="S48" s="50" t="s">
-        <v>126</v>
+        <v>198</v>
       </c>
       <c r="T48" s="50" t="s">
         <v>199</v>
@@ -18065,7 +17682,7 @@
       </c>
       <c r="AM48" s="49">
         <f t="shared" si="16"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AN48" s="49">
         <f t="shared" si="17"/>
@@ -19866,19 +19483,19 @@
         <v>223</v>
       </c>
       <c r="AC63" s="107" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="AD63" s="107" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AE63" s="107" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AF63" s="107" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="AG63" s="105" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="AH63" s="105" t="s">
         <v>223</v>
@@ -19895,15 +19512,15 @@
       </c>
       <c r="AM63" s="49">
         <f t="shared" si="16"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AN63" s="49">
         <f t="shared" si="17"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AO63" s="49">
         <f t="shared" si="18"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AP63" s="49">
         <f t="shared" si="19"/>
@@ -19991,10 +19608,10 @@
         <v>198</v>
       </c>
       <c r="AD64" s="107" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AE64" s="107" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="AF64" s="105" t="s">
         <v>222</v>
@@ -20017,7 +19634,7 @@
       </c>
       <c r="AM64" s="49">
         <f t="shared" si="16"/>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AN64" s="49">
         <f t="shared" si="17"/>
@@ -20025,7 +19642,7 @@
       </c>
       <c r="AO64" s="49">
         <f t="shared" si="18"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AP64" s="49">
         <f t="shared" si="19"/>
@@ -20113,7 +19730,7 @@
         <v>199</v>
       </c>
       <c r="AD65" s="107" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="AE65" s="105" t="s">
         <v>222</v>
@@ -20143,11 +19760,11 @@
       </c>
       <c r="AN65" s="49">
         <f t="shared" si="17"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AO65" s="49">
         <f t="shared" si="18"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AP65" s="49">
         <f t="shared" si="19"/>
@@ -20601,13 +20218,13 @@
         <v>223</v>
       </c>
       <c r="AD69" s="107" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="AE69" s="114" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AF69" s="114" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AG69" s="114" t="s">
         <v>222</v>
@@ -20627,11 +20244,11 @@
       </c>
       <c r="AM69" s="49">
         <f t="shared" si="16"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AN69" s="49">
         <f t="shared" si="17"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AO69" s="49">
         <f t="shared" si="18"/>
@@ -21339,7 +20956,7 @@
         <v>198</v>
       </c>
       <c r="AF75" s="114" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AG75" s="114" t="s">
         <v>199</v>
@@ -21359,11 +20976,11 @@
       </c>
       <c r="AM75" s="49">
         <f t="shared" si="16"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AN75" s="49">
         <f t="shared" si="17"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AO75" s="49">
         <f t="shared" si="18"/>
@@ -21969,15 +21586,15 @@
       </c>
       <c r="AM80" s="49">
         <f>COUNTIF($F63:$AJ63,"M*")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AN80" s="49">
         <f>COUNTIF($F63:$AJ63,"A*")</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AO80" s="49">
         <f>COUNTIF($F63:$AJ63,"N*")</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AP80" s="49">
         <f>COUNTIF($F63:$AJ63,"O*")</f>
@@ -22091,7 +21708,7 @@
       </c>
       <c r="AM81" s="49">
         <f t="shared" ref="AM81:AM98" si="20">COUNTIF($F64:$AJ64,"M*")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AN81" s="49">
         <f t="shared" ref="AN81:AN98" si="21">COUNTIF($F64:$AJ64,"A*")</f>
@@ -22099,7 +21716,7 @@
       </c>
       <c r="AO81" s="49">
         <f t="shared" ref="AO81:AO98" si="22">COUNTIF($F64:$AJ64,"N*")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AP81" s="49">
         <f t="shared" ref="AP81:AP98" si="23">COUNTIF($F64:$AJ64,"O*")</f>
@@ -22149,11 +21766,11 @@
       </c>
       <c r="AN82" s="49">
         <f t="shared" si="21"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AO82" s="49">
         <f t="shared" si="22"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AP82" s="49">
         <f t="shared" si="23"/>
@@ -22260,7 +21877,7 @@
       </c>
       <c r="AC83" s="37">
         <f t="shared" si="25"/>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AD83" s="37">
         <f t="shared" si="25"/>
@@ -22268,15 +21885,15 @@
       </c>
       <c r="AE83" s="37">
         <f t="shared" si="25"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AF83" s="37">
         <f t="shared" si="25"/>
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="AG83" s="37">
         <f t="shared" si="25"/>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AH83" s="37">
         <f t="shared" si="25"/>
@@ -22284,7 +21901,7 @@
       </c>
       <c r="AI83" s="37">
         <f t="shared" si="25"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AJ83" s="37">
         <f t="shared" si="25"/>
@@ -22395,19 +22012,19 @@
       </c>
       <c r="Y84" s="37">
         <f t="shared" si="26"/>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="Z84" s="37">
         <f t="shared" si="26"/>
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="AA84" s="37">
         <f t="shared" si="26"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="AB84" s="37">
         <f t="shared" si="26"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AC84" s="37">
         <f t="shared" si="26"/>
@@ -22415,19 +22032,19 @@
       </c>
       <c r="AD84" s="37">
         <f t="shared" si="26"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AE84" s="37">
         <f t="shared" si="26"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AF84" s="37">
         <f t="shared" si="26"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AG84" s="37">
         <f t="shared" si="26"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AH84" s="37">
         <f t="shared" si="26"/>
@@ -22506,15 +22123,15 @@
       </c>
       <c r="O85" s="37">
         <f t="shared" si="27"/>
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="P85" s="37">
         <f t="shared" si="27"/>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="Q85" s="37">
         <f t="shared" si="27"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="R85" s="37">
         <f t="shared" si="27"/>
@@ -22562,27 +22179,27 @@
       </c>
       <c r="AC85" s="37">
         <f t="shared" si="27"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AD85" s="37">
         <f t="shared" si="27"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AE85" s="37">
         <f t="shared" si="27"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AF85" s="37">
         <f t="shared" si="27"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AG85" s="37">
         <f t="shared" si="27"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AH85" s="37">
         <f t="shared" si="27"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AI85" s="37">
         <f t="shared" si="27"/>
@@ -22749,11 +22366,11 @@
       </c>
       <c r="AM86" s="49">
         <f t="shared" si="20"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AN86" s="49">
         <f t="shared" si="21"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AO86" s="49">
         <f t="shared" si="22"/>
@@ -23110,15 +22727,15 @@
       </c>
       <c r="O89" s="52">
         <f t="shared" si="31"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P89" s="52">
         <f t="shared" si="31"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q89" s="52">
         <f t="shared" si="31"/>
-        <v>-2</v>
+        <v>-3</v>
       </c>
       <c r="R89" s="52">
         <f t="shared" si="31"/>
@@ -23150,47 +22767,47 @@
       </c>
       <c r="Y89" s="52">
         <f t="shared" si="31"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="Z89" s="52">
         <f t="shared" si="31"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AA89" s="52">
         <f t="shared" si="31"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AB89" s="52">
         <f t="shared" si="31"/>
-        <v>0</v>
+        <v>-1</v>
       </c>
       <c r="AC89" s="52">
         <f t="shared" si="31"/>
-        <v>-1</v>
+        <v>-3</v>
       </c>
       <c r="AD89" s="52">
         <f t="shared" si="31"/>
-        <v>-5</v>
+        <v>-7</v>
       </c>
       <c r="AE89" s="52">
         <f t="shared" si="31"/>
-        <v>-5</v>
+        <v>-8</v>
       </c>
       <c r="AF89" s="52">
         <f t="shared" si="31"/>
-        <v>-5</v>
+        <v>-9</v>
       </c>
       <c r="AG89" s="52">
         <f t="shared" si="31"/>
-        <v>-5</v>
+        <v>-8</v>
       </c>
       <c r="AH89" s="52">
         <f t="shared" si="31"/>
-        <v>-10</v>
+        <v>-11</v>
       </c>
       <c r="AI89" s="52">
         <f t="shared" si="31"/>
-        <v>-6</v>
+        <v>-7</v>
       </c>
       <c r="AJ89" s="52">
         <f t="shared" si="31"/>
@@ -23317,15 +22934,15 @@
       </c>
       <c r="O91" s="41">
         <f t="shared" si="32"/>
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="P91" s="41">
         <f t="shared" si="32"/>
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="Q91" s="41">
         <f t="shared" si="32"/>
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="R91" s="41">
         <f t="shared" si="32"/>
@@ -23357,47 +22974,47 @@
       </c>
       <c r="Y91" s="41">
         <f t="shared" si="32"/>
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="Z91" s="41">
         <f t="shared" si="32"/>
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="AA91" s="41">
         <f t="shared" si="32"/>
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="AB91" s="41">
         <f t="shared" si="32"/>
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="AC91" s="41">
         <f t="shared" si="32"/>
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="AD91" s="41">
         <f t="shared" si="32"/>
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="AE91" s="41">
         <f t="shared" si="32"/>
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AF91" s="41">
         <f t="shared" si="32"/>
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="AG91" s="41">
         <f t="shared" si="32"/>
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="AH91" s="41">
         <f t="shared" si="32"/>
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="AI91" s="41">
         <f t="shared" si="32"/>
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="AJ91" s="41">
         <v>18</v>
@@ -23528,11 +23145,11 @@
       </c>
       <c r="AM92" s="49">
         <f t="shared" si="20"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AN92" s="49">
         <f t="shared" si="21"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AO92" s="49">
         <f t="shared" si="22"/>
@@ -23587,15 +23204,15 @@
       </c>
       <c r="O93" s="37">
         <f t="shared" si="33"/>
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="P93" s="37">
         <f t="shared" si="33"/>
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="Q93" s="37">
         <f t="shared" si="33"/>
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="R93" s="37">
         <f t="shared" si="33"/>
@@ -23627,47 +23244,47 @@
       </c>
       <c r="Y93" s="37">
         <f t="shared" si="33"/>
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="Z93" s="37">
         <f t="shared" si="33"/>
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="AA93" s="37">
         <f t="shared" si="33"/>
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="AB93" s="37">
         <f t="shared" si="33"/>
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="AC93" s="37">
         <f t="shared" si="33"/>
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="AD93" s="37">
         <f t="shared" si="33"/>
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="AE93" s="37">
         <f t="shared" si="33"/>
-        <v>53</v>
+        <v>50</v>
       </c>
       <c r="AF93" s="37">
         <f t="shared" si="33"/>
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="AG93" s="37">
         <f t="shared" si="33"/>
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="AH93" s="37">
         <f t="shared" si="33"/>
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="AI93" s="37">
         <f t="shared" si="33"/>
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="AJ93" s="37">
         <v>35</v>
@@ -24031,23 +23648,25 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ8">
-    <cfRule type="containsText" dxfId="42" priority="43" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="168" priority="112" operator="containsText" text="ME07">
+      <formula>NOT(ISERROR(SEARCH("ME07",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="167" priority="110" operator="containsText" text="AN13">
+      <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="166" priority="111" operator="containsText" text="OFF">
+      <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F5:AJ8">
+    <cfRule type="containsText" dxfId="165" priority="43" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="47" priority="44" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="164" priority="48" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="46" priority="45" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="163" priority="52" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="45" priority="46" operator="containsText" text="AN13">
-      <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="44" priority="47" operator="containsText" text="OFF">
-      <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="43" priority="48" operator="containsText" text="ME07">
-      <formula>NOT(ISERROR(SEARCH("ME07",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F63:AJ81">
@@ -26420,23 +26039,23 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ8">
-    <cfRule type="containsText" dxfId="90" priority="2" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="124" priority="1" operator="containsText" text="LV">
+      <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
+    </cfRule>
+    <cfRule type="containsText" dxfId="123" priority="2" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="91" priority="3" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="122" priority="3" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="92" priority="4" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="121" priority="4" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="93" priority="5" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="120" priority="5" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="94" priority="6" operator="containsText" text="ME07">
+    <cfRule type="containsText" dxfId="119" priority="6" operator="containsText" text="ME07">
       <formula>NOT(ISERROR(SEARCH("ME07",F5)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="95" priority="1" operator="containsText" text="LV">
-      <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -26930,16 +26549,16 @@
         <v>223</v>
       </c>
       <c r="AF6" s="50" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="AG6" s="50" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="AH6" s="50" t="s">
         <v>199</v>
       </c>
       <c r="AI6" s="50" t="s">
-        <v>199</v>
+        <v>222</v>
       </c>
       <c r="AJ6" s="50" t="s">
         <v>222</v>
@@ -26950,15 +26569,15 @@
       </c>
       <c r="AM6" s="49">
         <f t="shared" si="1"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AN6" s="49">
         <f t="shared" si="2"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AO6" s="49">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AP6" s="49">
         <f t="shared" si="4"/>
@@ -27049,19 +26668,19 @@
         <v>223</v>
       </c>
       <c r="AE7" s="50" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="AF7" s="50" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AG7" s="50" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AH7" s="50" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="AI7" s="50" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="AJ7" s="50" t="s">
         <v>223</v>
@@ -27072,15 +26691,15 @@
       </c>
       <c r="AM7" s="49">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AN7" s="49">
         <f t="shared" si="2"/>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AO7" s="49">
         <f t="shared" si="3"/>
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="AP7" s="49">
         <f t="shared" si="4"/>
@@ -27183,7 +26802,7 @@
         <v>198</v>
       </c>
       <c r="AI8" s="50" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AJ8" s="50" t="s">
         <v>199</v>
@@ -27194,11 +26813,11 @@
       </c>
       <c r="AM8" s="49">
         <f t="shared" si="1"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AN8" s="49">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AO8" s="49">
         <f t="shared" si="3"/>
@@ -27596,15 +27215,15 @@
       </c>
       <c r="AE12" s="37">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AF12" s="37">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AG12" s="37">
         <f t="shared" si="5"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH12" s="37">
         <f t="shared" si="5"/>
@@ -27612,7 +27231,7 @@
       </c>
       <c r="AI12" s="37">
         <f t="shared" si="5"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AJ12" s="37">
         <f t="shared" si="5"/>
@@ -27731,11 +27350,11 @@
       </c>
       <c r="AF13" s="37">
         <f t="shared" si="6"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AG13" s="37">
         <f t="shared" si="6"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AH13" s="37">
         <f t="shared" si="6"/>
@@ -27870,7 +27489,7 @@
       </c>
       <c r="AH14" s="37">
         <f t="shared" si="7"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AI14" s="37">
         <f t="shared" si="7"/>
@@ -28382,23 +28001,23 @@
       </c>
       <c r="AE18" s="51">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF18" s="51">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>-1</v>
       </c>
       <c r="AG18" s="51">
         <f t="shared" si="11"/>
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH18" s="51">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AI18" s="51">
         <f t="shared" si="11"/>
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AJ18" s="51">
         <f t="shared" si="11"/>
@@ -28549,23 +28168,23 @@
       </c>
       <c r="AE20" s="41">
         <f t="shared" si="12"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AF20" s="41">
         <f t="shared" si="12"/>
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="AG20" s="41">
         <f t="shared" si="12"/>
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="AH20" s="41">
         <f t="shared" si="12"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AI20" s="41">
         <f t="shared" si="12"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AJ20" s="41">
         <v>18</v>
@@ -28779,23 +28398,23 @@
       </c>
       <c r="AE22" s="37">
         <f t="shared" si="13"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AF22" s="37">
         <f t="shared" si="13"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AG22" s="37">
         <f t="shared" si="13"/>
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="AH22" s="37">
         <f t="shared" si="13"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AI22" s="37">
         <f t="shared" si="13"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AJ22" s="37">
         <v>35</v>
@@ -28963,34 +28582,34 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ10">
-    <cfRule type="containsText" dxfId="177" priority="1" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="118" priority="1" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="176" priority="2" operator="containsText" text="STNN21">
+    <cfRule type="containsText" dxfId="117" priority="2" operator="containsText" text="STNN21">
       <formula>NOT(ISERROR(SEARCH("STNN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="175" priority="3" operator="containsText" text="STAN13">
+    <cfRule type="containsText" dxfId="116" priority="3" operator="containsText" text="STAN13">
       <formula>NOT(ISERROR(SEARCH("STAN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="174" priority="4" operator="containsText" text="STMN06">
+    <cfRule type="containsText" dxfId="115" priority="4" operator="containsText" text="STMN06">
       <formula>NOT(ISERROR(SEARCH("STMN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="173" priority="5" operator="containsText" text="MN12">
+    <cfRule type="containsText" dxfId="114" priority="5" operator="containsText" text="MN12">
       <formula>NOT(ISERROR(SEARCH("MN12",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="172" priority="6" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="113" priority="6" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="171" priority="7" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="112" priority="7" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="170" priority="8" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="111" priority="8" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="169" priority="9" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="110" priority="9" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="168" priority="10" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="109" priority="10" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -29431,13 +29050,13 @@
         <v>198</v>
       </c>
       <c r="O6" s="50" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="P6" s="87" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="Q6" s="50" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="R6" s="50" t="s">
         <v>222</v>
@@ -29506,11 +29125,11 @@
       </c>
       <c r="AN6" s="49">
         <f t="shared" ref="AN6:AN19" si="2">COUNTIF($F6:$AJ6,"A*")</f>
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="AO6" s="49">
         <f t="shared" ref="AO6:AO19" si="3">COUNTIF($F6:$AJ6,"N*")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AP6" s="49">
         <f t="shared" ref="AP6:AP19" si="4">COUNTIF($F6:$AJ6,"O*")</f>
@@ -29675,7 +29294,7 @@
         <v>199</v>
       </c>
       <c r="O8" s="50" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="P8" s="50" t="s">
         <v>222</v>
@@ -29750,11 +29369,11 @@
       </c>
       <c r="AN8" s="49">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AO8" s="49">
         <f t="shared" si="3"/>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AP8" s="49">
         <f t="shared" si="4"/>
@@ -29830,7 +29449,7 @@
         <v>198</v>
       </c>
       <c r="Z9" s="50" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AA9" s="50" t="s">
         <v>199</v>
@@ -29868,11 +29487,11 @@
       </c>
       <c r="AM9" s="49">
         <f t="shared" si="1"/>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="AN9" s="49">
         <f t="shared" si="2"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AO9" s="49">
         <f t="shared" si="3"/>
@@ -29970,7 +29589,7 @@
         <v>198</v>
       </c>
       <c r="AF10" s="111" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AG10" s="111" t="s">
         <v>199</v>
@@ -29990,11 +29609,11 @@
       </c>
       <c r="AM10" s="49">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AN10" s="49">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AO10" s="49">
         <f t="shared" si="3"/>
@@ -30410,7 +30029,7 @@
         <v>199</v>
       </c>
       <c r="P14" s="50" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="Q14" s="50" t="s">
         <v>222</v>
@@ -30482,11 +30101,11 @@
       </c>
       <c r="AN14" s="49">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AO14" s="49">
         <f t="shared" si="3"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AP14" s="49">
         <f t="shared" si="4"/>
@@ -30681,19 +30300,19 @@
         <v>223</v>
       </c>
       <c r="Y16" s="50" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="Z16" s="50" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="AA16" s="50" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AB16" s="50" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AC16" s="87" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="AD16" s="87" t="s">
         <v>223</v>
@@ -30722,15 +30341,15 @@
       </c>
       <c r="AM16" s="49">
         <f>COUNTIF($F16:$AJ16,"M*")</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AN16" s="49">
         <f>COUNTIF($F16:$AJ16,"A*")</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AO16" s="49">
         <f>COUNTIF($F16:$AJ16,"N*")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AP16" s="49">
         <f>COUNTIF($F16:$AJ16,"O*")</f>
@@ -30803,7 +30422,7 @@
         <v>198</v>
       </c>
       <c r="Y17" s="50" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="Z17" s="50" t="s">
         <v>199</v>
@@ -30824,7 +30443,7 @@
         <v>198</v>
       </c>
       <c r="AF17" s="111" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AG17" s="111" t="s">
         <v>199</v>
@@ -30844,11 +30463,11 @@
       </c>
       <c r="AM17" s="49">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AN17" s="49">
         <f t="shared" si="2"/>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AO17" s="49">
         <f t="shared" si="3"/>
@@ -31352,19 +30971,19 @@
       </c>
       <c r="Y22" s="37">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Z22" s="37">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AA22" s="37">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AB22" s="37">
         <f t="shared" si="6"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AC22" s="37">
         <f t="shared" si="6"/>
@@ -31443,15 +31062,15 @@
       </c>
       <c r="O23" s="37">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P23" s="37">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="Q23" s="37">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R23" s="37">
         <f t="shared" si="7"/>
@@ -31499,7 +31118,7 @@
       </c>
       <c r="AC23" s="37">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AD23" s="37">
         <f t="shared" si="7"/>
@@ -31836,15 +31455,15 @@
       </c>
       <c r="O26" s="52">
         <f t="shared" si="10"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="P26" s="52">
         <f t="shared" si="10"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Q26" s="52">
         <f t="shared" si="10"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="R26" s="52">
         <f t="shared" si="10"/>
@@ -31876,23 +31495,23 @@
       </c>
       <c r="Y26" s="52">
         <f t="shared" si="10"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="Z26" s="52">
         <f t="shared" si="10"/>
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="AA26" s="52">
         <f t="shared" si="10"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AB26" s="52">
         <f t="shared" si="10"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AC26" s="52">
         <f t="shared" si="10"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AD26" s="52">
         <f t="shared" si="10"/>
@@ -32000,15 +31619,15 @@
       </c>
       <c r="O28" s="41">
         <f t="shared" si="11"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="P28" s="41">
         <f t="shared" si="11"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Q28" s="41">
         <f t="shared" si="11"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="R28" s="41">
         <f t="shared" si="11"/>
@@ -32040,23 +31659,23 @@
       </c>
       <c r="Y28" s="41">
         <f t="shared" si="11"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="Z28" s="41">
         <f t="shared" si="11"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AA28" s="41">
         <f t="shared" si="11"/>
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="AB28" s="41">
         <f t="shared" si="11"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AC28" s="41">
         <f t="shared" si="11"/>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="AD28" s="41">
         <f t="shared" si="11"/>
@@ -32230,15 +31849,15 @@
       </c>
       <c r="O30" s="37">
         <f t="shared" si="12"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="P30" s="37">
         <f t="shared" si="12"/>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Q30" s="37">
         <f t="shared" si="12"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="R30" s="37">
         <f t="shared" si="12"/>
@@ -32270,23 +31889,23 @@
       </c>
       <c r="Y30" s="37">
         <f t="shared" si="12"/>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="Z30" s="37">
         <f t="shared" si="12"/>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AA30" s="37">
         <f t="shared" si="12"/>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AB30" s="37">
         <f t="shared" si="12"/>
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="AC30" s="37">
         <f t="shared" si="12"/>
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="AD30" s="37">
         <f t="shared" si="12"/>
@@ -32430,40 +32049,40 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ19">
-    <cfRule type="containsText" dxfId="167" priority="1" operator="containsText" text="STMN06">
+    <cfRule type="containsText" dxfId="108" priority="1" operator="containsText" text="STMN06">
       <formula>NOT(ISERROR(SEARCH("STMN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="166" priority="3" operator="containsText" text="STAN13">
+    <cfRule type="containsText" dxfId="107" priority="3" operator="containsText" text="STAN13">
       <formula>NOT(ISERROR(SEARCH("STAN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="165" priority="4" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="106" priority="4" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="164" priority="5" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="105" priority="5" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="163" priority="6" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="104" priority="6" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="162" priority="7" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="103" priority="7" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="161" priority="8" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="102" priority="8" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="160" priority="9" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="101" priority="9" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="159" priority="10" operator="containsText" text="STAN13">
+    <cfRule type="containsText" dxfId="100" priority="10" operator="containsText" text="STAN13">
       <formula>NOT(ISERROR(SEARCH("STAN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="158" priority="11" operator="containsText" text="STNN21">
+    <cfRule type="containsText" dxfId="99" priority="11" operator="containsText" text="STNN21">
       <formula>NOT(ISERROR(SEARCH("STNN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="157" priority="12" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="98" priority="12" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="156" priority="13" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="97" priority="13" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -34136,10 +33755,10 @@
         <v>223</v>
       </c>
       <c r="R16" s="50" t="s">
-        <v>198</v>
+        <v>126</v>
       </c>
       <c r="S16" s="50" t="s">
-        <v>198</v>
+        <v>126</v>
       </c>
       <c r="T16" s="50" t="s">
         <v>199</v>
@@ -34198,7 +33817,7 @@
       </c>
       <c r="AM16" s="49">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AN16" s="49">
         <f t="shared" si="2"/>
@@ -34990,10 +34609,10 @@
         <v>223</v>
       </c>
       <c r="R23" s="50" t="s">
-        <v>126</v>
+        <v>198</v>
       </c>
       <c r="S23" s="50" t="s">
-        <v>126</v>
+        <v>198</v>
       </c>
       <c r="T23" s="50" t="s">
         <v>199</v>
@@ -35052,7 +34671,7 @@
       </c>
       <c r="AM23" s="49">
         <f t="shared" si="1"/>
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="AN23" s="49">
         <f t="shared" si="2"/>
@@ -38286,34 +37905,34 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ37">
-    <cfRule type="containsText" dxfId="155" priority="1" operator="containsText" text="MN12">
+    <cfRule type="containsText" dxfId="96" priority="1" operator="containsText" text="MN12">
       <formula>NOT(ISERROR(SEARCH("MN12",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="154" priority="2" operator="containsText" text="STNN21">
+    <cfRule type="containsText" dxfId="95" priority="2" operator="containsText" text="STNN21">
       <formula>NOT(ISERROR(SEARCH("STNN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="153" priority="3" operator="containsText" text="STAN13">
+    <cfRule type="containsText" dxfId="94" priority="3" operator="containsText" text="STAN13">
       <formula>NOT(ISERROR(SEARCH("STAN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="152" priority="4" operator="containsText" text="STMN06">
+    <cfRule type="containsText" dxfId="93" priority="4" operator="containsText" text="STMN06">
       <formula>NOT(ISERROR(SEARCH("STMN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="151" priority="5" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="92" priority="5" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="150" priority="6" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="91" priority="6" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="149" priority="7" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="90" priority="7" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="148" priority="8" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="89" priority="8" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="147" priority="9" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="88" priority="9" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="146" priority="10" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="87" priority="10" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -38674,19 +38293,19 @@
         <v>223</v>
       </c>
       <c r="AC5" s="107" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="AD5" s="107" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AE5" s="107" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AF5" s="107" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="AG5" s="105" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="AH5" s="105" t="s">
         <v>223</v>
@@ -38703,15 +38322,15 @@
       </c>
       <c r="AM5" s="22">
         <f>COUNTIF($F5:$AJ5,"M*")</f>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AN5" s="22">
         <f>COUNTIF($F5:$AJ5,"A*")</f>
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="AO5" s="22">
         <f>COUNTIF($F5:$AJ5,"N*")</f>
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="AP5" s="22">
         <f>COUNTIF($F5:$AJ5,"O*")</f>
@@ -38799,10 +38418,10 @@
         <v>198</v>
       </c>
       <c r="AD6" s="107" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="AE6" s="107" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="AF6" s="105" t="s">
         <v>222</v>
@@ -38825,7 +38444,7 @@
       </c>
       <c r="AM6" s="22">
         <f t="shared" ref="AM6:AM23" si="1">COUNTIF($F6:$AJ6,"M*")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="AN6" s="22">
         <f t="shared" ref="AN6:AN23" si="2">COUNTIF($F6:$AJ6,"A*")</f>
@@ -38833,7 +38452,7 @@
       </c>
       <c r="AO6" s="22">
         <f t="shared" ref="AO6:AO23" si="3">COUNTIF($F6:$AJ6,"N*")</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="AP6" s="22">
         <f t="shared" ref="AP6:AP23" si="4">COUNTIF($F6:$AJ6,"O*")</f>
@@ -38921,7 +38540,7 @@
         <v>199</v>
       </c>
       <c r="AD7" s="107" t="s">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="AE7" s="105" t="s">
         <v>222</v>
@@ -38951,11 +38570,11 @@
       </c>
       <c r="AN7" s="22">
         <f t="shared" si="2"/>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="AO7" s="22">
         <f t="shared" si="3"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AP7" s="22">
         <f t="shared" si="4"/>
@@ -39409,13 +39028,13 @@
         <v>223</v>
       </c>
       <c r="AD11" s="107" t="s">
-        <v>198</v>
+        <v>224</v>
       </c>
       <c r="AE11" s="114" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AF11" s="114" t="s">
-        <v>199</v>
+        <v>224</v>
       </c>
       <c r="AG11" s="114" t="s">
         <v>222</v>
@@ -39435,11 +39054,11 @@
       </c>
       <c r="AM11" s="22">
         <f t="shared" si="1"/>
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="AN11" s="22">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="AO11" s="22">
         <f t="shared" si="3"/>
@@ -40147,7 +39766,7 @@
         <v>198</v>
       </c>
       <c r="AF17" s="114" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="AG17" s="114" t="s">
         <v>199</v>
@@ -40167,11 +39786,11 @@
       </c>
       <c r="AM17" s="22">
         <f t="shared" si="1"/>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="AN17" s="22">
         <f t="shared" si="2"/>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="AO17" s="22">
         <f t="shared" si="3"/>
@@ -41048,7 +40667,7 @@
       </c>
       <c r="AC25" s="37">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AD25" s="37">
         <f t="shared" si="5"/>
@@ -41060,7 +40679,7 @@
       </c>
       <c r="AF25" s="37">
         <f t="shared" si="5"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AG25" s="37">
         <f t="shared" si="5"/>
@@ -41183,11 +40802,11 @@
       </c>
       <c r="AD26" s="37">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE26" s="37">
         <f t="shared" si="6"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AF26" s="37">
         <f t="shared" si="6"/>
@@ -41314,19 +40933,19 @@
       </c>
       <c r="AD27" s="37">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AE27" s="37">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AF27" s="37">
         <f t="shared" si="7"/>
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="AG27" s="37">
         <f t="shared" si="7"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AH27" s="37">
         <f t="shared" si="7"/>
@@ -41834,23 +41453,23 @@
       </c>
       <c r="AC31" s="39">
         <f t="shared" si="12"/>
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="AD31" s="39">
         <f t="shared" si="12"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AE31" s="39">
         <f t="shared" si="12"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AF31" s="39">
         <f t="shared" si="12"/>
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="AG31" s="39">
         <f t="shared" si="12"/>
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AH31" s="39">
         <f t="shared" si="12"/>
@@ -42001,23 +41620,23 @@
       </c>
       <c r="AC33" s="41">
         <f t="shared" si="13"/>
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="AD33" s="41">
         <f t="shared" si="13"/>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="AE33" s="41">
         <f t="shared" si="13"/>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="AF33" s="41">
         <f t="shared" si="13"/>
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="AG33" s="41">
         <f t="shared" si="13"/>
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="AH33" s="41">
         <f t="shared" si="13"/>
@@ -42232,23 +41851,23 @@
       </c>
       <c r="AC35" s="37">
         <f t="shared" si="14"/>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="AD35" s="37">
         <f t="shared" si="14"/>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AE35" s="37">
         <f t="shared" si="14"/>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AF35" s="37">
         <f t="shared" si="14"/>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="AG35" s="37">
         <f t="shared" si="14"/>
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="AH35" s="37">
         <f t="shared" si="14"/>
@@ -42381,34 +42000,34 @@
   </mergeCells>
   <phoneticPr fontId="14" type="noConversion"/>
   <conditionalFormatting sqref="F5:AJ23">
-    <cfRule type="containsText" dxfId="145" priority="1" operator="containsText" text="STMN06">
+    <cfRule type="containsText" dxfId="86" priority="1" operator="containsText" text="STMN06">
       <formula>NOT(ISERROR(SEARCH("STMN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="144" priority="2" operator="containsText" text="STAN13">
+    <cfRule type="containsText" dxfId="85" priority="2" operator="containsText" text="STAN13">
       <formula>NOT(ISERROR(SEARCH("STAN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="143" priority="3" operator="containsText" text="STNN21">
+    <cfRule type="containsText" dxfId="84" priority="3" operator="containsText" text="STNN21">
       <formula>NOT(ISERROR(SEARCH("STNN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="142" priority="4" operator="containsText" text="LV">
+    <cfRule type="containsText" dxfId="83" priority="4" operator="containsText" text="LV">
       <formula>NOT(ISERROR(SEARCH("LV",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="141" priority="5" operator="containsText" text="TR">
+    <cfRule type="containsText" dxfId="82" priority="5" operator="containsText" text="TR">
       <formula>NOT(ISERROR(SEARCH("TR",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="140" priority="6" operator="containsText" text="NN21">
+    <cfRule type="containsText" dxfId="81" priority="6" operator="containsText" text="NN21">
       <formula>NOT(ISERROR(SEARCH("NN21",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="139" priority="7" operator="containsText" text="NN13">
+    <cfRule type="containsText" dxfId="80" priority="7" operator="containsText" text="NN13">
       <formula>NOT(ISERROR(SEARCH("NN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="138" priority="8" operator="containsText" text="AN13">
+    <cfRule type="containsText" dxfId="79" priority="8" operator="containsText" text="AN13">
       <formula>NOT(ISERROR(SEARCH("AN13",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="137" priority="9" operator="containsText" text="MN06">
+    <cfRule type="containsText" dxfId="78" priority="9" operator="containsText" text="MN06">
       <formula>NOT(ISERROR(SEARCH("MN06",F5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="136" priority="10" operator="containsText" text="OFF">
+    <cfRule type="containsText" dxfId="77" priority="10" operator="containsText" text="OFF">
       <formula>NOT(ISERROR(SEARCH("OFF",F5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -45183,117 +44802,117 @@
     <mergeCell ref="B8:C8"/>
   </mergeCells>
   <conditionalFormatting sqref="E5:AH10">
-    <cfRule type="containsText" dxfId="135" priority="23" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="76" priority="23" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="134" priority="24" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="75" priority="24" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="133" priority="25" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="74" priority="25" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="132" priority="26" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="73" priority="26" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="131" priority="27" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="72" priority="27" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="130" priority="28" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="71" priority="28" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="129" priority="29" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="70" priority="29" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="128" priority="30" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="69" priority="30" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E5:AH15">
-    <cfRule type="containsText" dxfId="127" priority="19" operator="containsText" text="A">
+    <cfRule type="containsText" dxfId="68" priority="19" operator="containsText" text="A">
       <formula>NOT(ISERROR(SEARCH("A",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="126" priority="5" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="67" priority="5" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E11:AH15">
-    <cfRule type="containsText" dxfId="125" priority="16" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="66" priority="16" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="124" priority="17" operator="containsText" text="O">
+    <cfRule type="containsText" dxfId="65" priority="17" operator="containsText" text="O">
       <formula>NOT(ISERROR(SEARCH("O",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="123" priority="18" operator="containsText" text="N">
+    <cfRule type="containsText" dxfId="64" priority="18" operator="containsText" text="N">
       <formula>NOT(ISERROR(SEARCH("N",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="122" priority="6" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="63" priority="6" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="121" priority="7" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="62" priority="7" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="120" priority="8" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="61" priority="8" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="119" priority="9" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="60" priority="9" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="118" priority="10" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="59" priority="10" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="117" priority="11" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="58" priority="11" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="116" priority="12" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="57" priority="12" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="115" priority="13" operator="containsText" text="STM">
+    <cfRule type="containsText" dxfId="56" priority="13" operator="containsText" text="STM">
       <formula>NOT(ISERROR(SEARCH("STM",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="114" priority="14" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="55" priority="14" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="113" priority="15" operator="containsText" text="STA">
+    <cfRule type="containsText" dxfId="54" priority="15" operator="containsText" text="STA">
       <formula>NOT(ISERROR(SEARCH("STA",E11)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="112" priority="20" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="53" priority="20" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E11)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E5:AI15">
-    <cfRule type="containsText" dxfId="111" priority="3" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="52" priority="3" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="110" priority="4" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="51" priority="4" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="109" priority="1" operator="containsText" text="STN">
+    <cfRule type="containsText" dxfId="50" priority="1" operator="containsText" text="STN">
       <formula>NOT(ISERROR(SEARCH("STN",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="108" priority="2" operator="containsText" text="STA">
+    <cfRule type="containsText" dxfId="49" priority="2" operator="containsText" text="STA">
       <formula>NOT(ISERROR(SEARCH("STA",E5)))</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F5:AH5 E6:AH10">
-    <cfRule type="containsText" dxfId="107" priority="31" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="48" priority="31" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="106" priority="32" operator="containsText" text="STA">
+    <cfRule type="containsText" dxfId="47" priority="32" operator="containsText" text="STA">
       <formula>NOT(ISERROR(SEARCH("STA",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="105" priority="33" operator="containsText" text="STM1">
+    <cfRule type="containsText" dxfId="46" priority="33" operator="containsText" text="STM1">
       <formula>NOT(ISERROR(SEARCH("STM1",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="104" priority="34" operator="containsText" text="O">
+    <cfRule type="containsText" dxfId="45" priority="34" operator="containsText" text="O">
       <formula>NOT(ISERROR(SEARCH("O",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="103" priority="35" operator="containsText" text="N">
+    <cfRule type="containsText" dxfId="44" priority="35" operator="containsText" text="N">
       <formula>NOT(ISERROR(SEARCH("N",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="102" priority="36" operator="containsText" text="A">
+    <cfRule type="containsText" dxfId="43" priority="36" operator="containsText" text="A">
       <formula>NOT(ISERROR(SEARCH("A",E5)))</formula>
     </cfRule>
-    <cfRule type="containsText" dxfId="101" priority="37" operator="containsText" text="M">
+    <cfRule type="containsText" dxfId="42" priority="37" operator="containsText" text="M">
       <formula>NOT(ISERROR(SEARCH("M",E5)))</formula>
     </cfRule>
   </conditionalFormatting>
@@ -45333,6 +44952,16 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_activity xmlns="0ecd8b7c-869e-4f04-a6a3-066c3c63b311" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="مستند" ma:contentTypeID="0x01010053585A714B17B949862FA1B71BD97610" ma:contentTypeVersion="20" ma:contentTypeDescription="إنشاء مستند جديد." ma:contentTypeScope="" ma:versionID="dd8bd6d392f178541f6ccf1c351709a2">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns1="http://schemas.microsoft.com/sharepoint/v3" xmlns:ns3="f1e9c892-1499-41bb-8a64-60ef909d8682" xmlns:ns4="0ecd8b7c-869e-4f04-a6a3-066c3c63b311" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="9f246d41c9a2b9a4922388dcb99eeb28" ns1:_="" ns3:_="" ns4:_="">
     <xsd:import namespace="http://schemas.microsoft.com/sharepoint/v3"/>
@@ -45602,7 +45231,7 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
   <Display>DocumentLibraryForm</Display>
@@ -45611,17 +45240,25 @@
 </FormTemplates>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_activity xmlns="0ecd8b7c-869e-4f04-a6a3-066c3c63b311" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04335F04-3ECE-4043-846B-35335B1D83ED}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="0ecd8b7c-869e-4f04-a6a3-066c3c63b311"/>
+    <ds:schemaRef ds:uri="f1e9c892-1499-41bb-8a64-60ef909d8682"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57D06F05-5672-4668-89C3-4F6754D4BC82}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -45641,28 +45278,10 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{D7131BC6-00FD-4253-878E-994124306B86}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{04335F04-3ECE-4043-846B-35335B1D83ED}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="0ecd8b7c-869e-4f04-a6a3-066c3c63b311"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="f1e9c892-1499-41bb-8a64-60ef909d8682"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>